<commit_message>
Sending to managers with ccs
</commit_message>
<xml_diff>
--- a/sheet/8462.xlsx
+++ b/sheet/8462.xlsx
@@ -874,10 +874,10 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>4.95</v>
+        <v>10.47</v>
       </c>
       <c r="H13" t="n">
-        <v>4.95</v>
+        <v>10.47</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>4.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="H25" t="n">
-        <v>4.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1354,10 +1354,10 @@
         <v>63</v>
       </c>
       <c r="C2" t="n">
-        <v>75.19</v>
+        <v>80.70999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>12.19</v>
+        <v>17.71</v>
       </c>
     </row>
     <row r="3">
@@ -1370,10 +1370,10 @@
         <v>54</v>
       </c>
       <c r="C3" t="n">
-        <v>62.13</v>
+        <v>66.53</v>
       </c>
       <c r="D3" t="n">
-        <v>8.130000000000001</v>
+        <v>12.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Yes signal with ms.rachel
</commit_message>
<xml_diff>
--- a/sheet/8462.xlsx
+++ b/sheet/8462.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,7 +470,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>403</v>
+        <v>1147</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>404</v>
+        <v>1148</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -540,7 +540,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>405</v>
+        <v>1149</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>406</v>
+        <v>1150</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>407</v>
+        <v>1151</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>408</v>
+        <v>1152</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -690,7 +690,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>409</v>
+        <v>1153</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>410</v>
+        <v>1154</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>411</v>
+        <v>1155</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>412</v>
+        <v>1156</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -830,7 +830,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>413</v>
+        <v>1157</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -840,14 +840,24 @@
       <c r="C12" s="2" t="n">
         <v>46153</v>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>07:00 PM</t>
+        </is>
+      </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>10.5</v>
       </c>
       <c r="G12" t="n">
         <v>9.74</v>
       </c>
       <c r="H12" t="n">
-        <v>9.74</v>
+        <v>-0.76</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -860,7 +870,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>414</v>
+        <v>1158</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -870,14 +880,24 @@
       <c r="C13" s="2" t="n">
         <v>46154</v>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>07:00 PM</t>
+        </is>
+      </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>10.5</v>
       </c>
       <c r="G13" t="n">
         <v>10.47</v>
       </c>
       <c r="H13" t="n">
-        <v>10.47</v>
+        <v>-0.03</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -890,34 +910,34 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>744</v>
+        <v>1159</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
+          <t>ESPINO, DAN A [0165]</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>46143</v>
+        <v>46155</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>06:30 PM</t>
+          <t>07:00 PM</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9</v>
+        <v>10.5</v>
       </c>
       <c r="G14" t="n">
-        <v>8.51</v>
+        <v>10.5</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.49</v>
+        <v>0</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -930,24 +950,34 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>745</v>
+        <v>1160</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
+          <t>ESPINO, DAN A [0165]</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>46144</v>
+        <v>46156</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>07:00 PM</t>
+        </is>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>10.5</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -960,24 +990,34 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>746</v>
+        <v>1161</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
+          <t>ESPINO, DAN A [0165]</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>46145</v>
+        <v>46157</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>07:00 PM</t>
+        </is>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>10.5</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>10.59</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -990,34 +1030,24 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>747</v>
+        <v>1162</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
+          <t>ESPINO, DAN A [0165]</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
+        <v>46158</v>
       </c>
       <c r="F17" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>8.9</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1030,34 +1060,24 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>748</v>
+        <v>1163</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
+          <t>ESPINO, DAN A [0165]</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>46147</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
+        <v>46159</v>
       </c>
       <c r="F18" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>9.23</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1070,34 +1090,34 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>749</v>
+        <v>1164</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
+          <t>ESPINO, DAN A [0165]</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>46148</v>
+        <v>46160</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>06:30 PM</t>
+          <t>07:00 PM</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>9</v>
+        <v>10.5</v>
       </c>
       <c r="G19" t="n">
-        <v>8.58</v>
+        <v>10.07</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.42</v>
+        <v>-0.43</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1110,34 +1130,34 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>750</v>
+        <v>1165</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
+          <t>ESPINO, DAN A [0165]</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>46149</v>
+        <v>46161</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>06:30 PM</t>
+          <t>07:00 PM</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>9</v>
+        <v>10.5</v>
       </c>
       <c r="G20" t="n">
-        <v>8.6</v>
+        <v>10.5</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.4</v>
+        <v>0</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1150,34 +1170,34 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>751</v>
+        <v>1166</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
+          <t>ESPINO, DAN A [0165]</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>46150</v>
+        <v>46162</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>06:30 PM</t>
+          <t>07:00 PM</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>9</v>
+        <v>10.5</v>
       </c>
       <c r="G21" t="n">
-        <v>6.1</v>
+        <v>4.92</v>
       </c>
       <c r="H21" t="n">
-        <v>-2.9</v>
+        <v>-5.58</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1190,7 +1210,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>752</v>
+        <v>2201</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1198,16 +1218,26 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>46151</v>
+        <v>46143</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>8.51</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>-0.49</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1220,7 +1250,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>753</v>
+        <v>2202</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1228,7 +1258,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>46152</v>
+        <v>46144</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -1250,7 +1280,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>754</v>
+        <v>2203</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1258,16 +1288,16 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>46153</v>
+        <v>46145</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>8.06</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>8.06</v>
+        <v>0</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1280,7 +1310,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>755</v>
+        <v>2204</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1288,23 +1318,633 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>9</v>
+      </c>
+      <c r="G25" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2205</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>46147</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>9</v>
+      </c>
+      <c r="G26" t="n">
+        <v>9.23</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2206</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>9</v>
+      </c>
+      <c r="G27" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-0.42</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2207</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>46149</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>9</v>
+      </c>
+      <c r="G28" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2208</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>46150</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>9</v>
+      </c>
+      <c r="G29" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-2.9</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2209</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>46151</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2210</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>46152</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2211</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>46153</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>9</v>
+      </c>
+      <c r="G32" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="H32" t="n">
+        <v>-0.9399999999999999</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2212</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
         <v>46154</v>
       </c>
-      <c r="F25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" t="n">
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>9</v>
+      </c>
+      <c r="G33" t="n">
         <v>8.550000000000001</v>
       </c>
-      <c r="H25" t="n">
+      <c r="H33" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2213</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>46155</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>9</v>
+      </c>
+      <c r="G34" t="n">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="H34" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2214</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>46156</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>9</v>
+      </c>
+      <c r="G35" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="H35" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2215</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>46157</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>9</v>
+      </c>
+      <c r="G36" t="n">
+        <v>8.48</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>2216</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>46158</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>2217</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>46159</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>2218</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>9</v>
+      </c>
+      <c r="G39" t="n">
         <v>8.550000000000001</v>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J25" t="n">
+      <c r="H39" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2219</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>46161</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>9</v>
+      </c>
+      <c r="G40" t="n">
+        <v>8.619999999999999</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>8462</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2220</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>NALBANDIAN, KARNIG [1407]</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>9</v>
+      </c>
+      <c r="G41" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
         <v>8462</v>
       </c>
     </row>
@@ -1351,13 +1991,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>63</v>
+        <v>147</v>
       </c>
       <c r="C2" t="n">
-        <v>80.70999999999999</v>
+        <v>137.29</v>
       </c>
       <c r="D2" t="n">
-        <v>17.71</v>
+        <v>-9.710000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -1367,13 +2007,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>54</v>
+        <v>126</v>
       </c>
       <c r="C3" t="n">
-        <v>66.53</v>
+        <v>113.04</v>
       </c>
       <c r="D3" t="n">
-        <v>12.53</v>
+        <v>-12.96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Yes signal with ms.rachel"
This reverts commit 44fe4e5d7b298fc4835ffecd58a4873c259ebb38.
</commit_message>
<xml_diff>
--- a/sheet/8462.xlsx
+++ b/sheet/8462.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,7 +470,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1147</v>
+        <v>403</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1148</v>
+        <v>404</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -540,7 +540,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1149</v>
+        <v>405</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1150</v>
+        <v>406</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1151</v>
+        <v>407</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1152</v>
+        <v>408</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -690,7 +690,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1153</v>
+        <v>409</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1154</v>
+        <v>410</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1155</v>
+        <v>411</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1156</v>
+        <v>412</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -830,7 +830,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1157</v>
+        <v>413</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -840,24 +840,14 @@
       <c r="C12" s="2" t="n">
         <v>46153</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>08:00 AM</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>07:00 PM</t>
-        </is>
-      </c>
       <c r="F12" t="n">
-        <v>10.5</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
         <v>9.74</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.76</v>
+        <v>9.74</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -870,7 +860,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1158</v>
+        <v>414</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -880,24 +870,14 @@
       <c r="C13" s="2" t="n">
         <v>46154</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>08:00 AM</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>07:00 PM</t>
-        </is>
-      </c>
       <c r="F13" t="n">
-        <v>10.5</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
         <v>10.47</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.03</v>
+        <v>10.47</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -910,34 +890,34 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1159</v>
+        <v>744</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ESPINO, DAN A [0165]</t>
+          <t>NALBANDIAN, KARNIG [1407]</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>46155</v>
+        <v>46143</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>07:00 PM</t>
+          <t>06:30 PM</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="G14" t="n">
-        <v>10.5</v>
+        <v>8.51</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>-0.49</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -950,34 +930,24 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1160</v>
+        <v>745</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ESPINO, DAN A [0165]</t>
+          <t>NALBANDIAN, KARNIG [1407]</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>46156</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>08:00 AM</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>07:00 PM</t>
-        </is>
+        <v>46144</v>
       </c>
       <c r="F15" t="n">
-        <v>10.5</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -990,34 +960,24 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1161</v>
+        <v>746</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ESPINO, DAN A [0165]</t>
+          <t>NALBANDIAN, KARNIG [1407]</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>46157</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>08:00 AM</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>07:00 PM</t>
-        </is>
+        <v>46145</v>
       </c>
       <c r="F16" t="n">
-        <v>10.5</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>10.59</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1030,24 +990,34 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1162</v>
+        <v>747</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ESPINO, DAN A [0165]</t>
+          <t>NALBANDIAN, KARNIG [1407]</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>46158</v>
+        <v>46146</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>8.9</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1060,24 +1030,34 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1163</v>
+        <v>748</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ESPINO, DAN A [0165]</t>
+          <t>NALBANDIAN, KARNIG [1407]</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>46159</v>
+        <v>46147</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>09:00 AM</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>9.23</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>0.23</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1090,34 +1070,34 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1164</v>
+        <v>749</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ESPINO, DAN A [0165]</t>
+          <t>NALBANDIAN, KARNIG [1407]</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>46160</v>
+        <v>46148</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>07:00 PM</t>
+          <t>06:30 PM</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="G19" t="n">
-        <v>10.07</v>
+        <v>8.58</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.43</v>
+        <v>-0.42</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1130,34 +1110,34 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1165</v>
+        <v>750</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ESPINO, DAN A [0165]</t>
+          <t>NALBANDIAN, KARNIG [1407]</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>46161</v>
+        <v>46149</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>07:00 PM</t>
+          <t>06:30 PM</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="G20" t="n">
-        <v>10.5</v>
+        <v>8.6</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>-0.4</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1170,34 +1150,34 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1166</v>
+        <v>751</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ESPINO, DAN A [0165]</t>
+          <t>NALBANDIAN, KARNIG [1407]</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>46162</v>
+        <v>46150</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>07:00 PM</t>
+          <t>06:30 PM</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="G21" t="n">
-        <v>4.92</v>
+        <v>6.1</v>
       </c>
       <c r="H21" t="n">
-        <v>-5.58</v>
+        <v>-2.9</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1210,7 +1190,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2201</v>
+        <v>752</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1218,26 +1198,16 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>46143</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
+        <v>46151</v>
       </c>
       <c r="F22" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>8.51</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>-0.49</v>
+        <v>0</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1250,7 +1220,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2202</v>
+        <v>753</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1258,7 +1228,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>46144</v>
+        <v>46152</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -1280,7 +1250,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2203</v>
+        <v>754</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1288,16 +1258,16 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>46145</v>
+        <v>46153</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>8.06</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>8.06</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1310,7 +1280,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2204</v>
+        <v>755</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1318,26 +1288,16 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
+        <v>46154</v>
       </c>
       <c r="F25" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>8.9</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.1</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1345,606 +1305,6 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>2205</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>46147</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>9</v>
-      </c>
-      <c r="G26" t="n">
-        <v>9.23</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J26" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>2206</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>46148</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>9</v>
-      </c>
-      <c r="G27" t="n">
-        <v>8.58</v>
-      </c>
-      <c r="H27" t="n">
-        <v>-0.42</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J27" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>2207</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>46149</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>9</v>
-      </c>
-      <c r="G28" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="H28" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J28" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>2208</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="n">
-        <v>46150</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>9</v>
-      </c>
-      <c r="G29" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="H29" t="n">
-        <v>-2.9</v>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J29" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>2209</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>46151</v>
-      </c>
-      <c r="F30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J30" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>2210</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>46152</v>
-      </c>
-      <c r="F31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J31" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>2211</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>46153</v>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>9</v>
-      </c>
-      <c r="G32" t="n">
-        <v>8.06</v>
-      </c>
-      <c r="H32" t="n">
-        <v>-0.9399999999999999</v>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J32" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>2212</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="n">
-        <v>46154</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>9</v>
-      </c>
-      <c r="G33" t="n">
-        <v>8.550000000000001</v>
-      </c>
-      <c r="H33" t="n">
-        <v>-0.45</v>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J33" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>2213</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>46155</v>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>9</v>
-      </c>
-      <c r="G34" t="n">
-        <v>8.529999999999999</v>
-      </c>
-      <c r="H34" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J34" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>2214</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>46156</v>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>9</v>
-      </c>
-      <c r="G35" t="n">
-        <v>8.23</v>
-      </c>
-      <c r="H35" t="n">
-        <v>-0.77</v>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J35" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>2215</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="n">
-        <v>46157</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>9</v>
-      </c>
-      <c r="G36" t="n">
-        <v>8.48</v>
-      </c>
-      <c r="H36" t="n">
-        <v>-0.52</v>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J36" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>2216</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>46158</v>
-      </c>
-      <c r="F37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J37" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>2217</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>46159</v>
-      </c>
-      <c r="F38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J38" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>2218</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>46160</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>9</v>
-      </c>
-      <c r="G39" t="n">
-        <v>8.550000000000001</v>
-      </c>
-      <c r="H39" t="n">
-        <v>-0.45</v>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J39" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>2219</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>46161</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>9</v>
-      </c>
-      <c r="G40" t="n">
-        <v>8.619999999999999</v>
-      </c>
-      <c r="H40" t="n">
-        <v>-0.38</v>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J40" t="n">
-        <v>8462</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>2220</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>NALBANDIAN, KARNIG [1407]</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="n">
-        <v>46162</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>09:00 AM</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>06:30 PM</t>
-        </is>
-      </c>
-      <c r="F41" t="n">
-        <v>9</v>
-      </c>
-      <c r="G41" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="H41" t="n">
-        <v>-4.9</v>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>ADMIN</t>
-        </is>
-      </c>
-      <c r="J41" t="n">
         <v>8462</v>
       </c>
     </row>
@@ -1991,13 +1351,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>147</v>
+        <v>63</v>
       </c>
       <c r="C2" t="n">
-        <v>137.29</v>
+        <v>80.70999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>-9.710000000000001</v>
+        <v>17.71</v>
       </c>
     </row>
     <row r="3">
@@ -2007,13 +1367,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>126</v>
+        <v>54</v>
       </c>
       <c r="C3" t="n">
-        <v>113.04</v>
+        <v>66.53</v>
       </c>
       <c r="D3" t="n">
-        <v>-12.96</v>
+        <v>12.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>